<commit_message>
Add data cleaning, analysis, and visualization projects with SQL and Python scripts
</commit_message>
<xml_diff>
--- a/Project1/Cleaned_Dataset.xlsx
+++ b/Project1/Cleaned_Dataset.xlsx
@@ -2969,7 +2969,7 @@
         </is>
       </c>
       <c r="N41" t="n">
-        <v>769.3799999999999</v>
+        <v>769.38</v>
       </c>
     </row>
     <row r="42">
@@ -4643,7 +4643,7 @@
         </is>
       </c>
       <c r="N68" t="n">
-        <v>635.9000000000001</v>
+        <v>635.9</v>
       </c>
     </row>
     <row r="69">
@@ -5821,7 +5821,7 @@
         </is>
       </c>
       <c r="N87" t="n">
-        <v>440.1899999999999</v>
+        <v>440.19</v>
       </c>
     </row>
     <row r="88">
@@ -7433,7 +7433,7 @@
         </is>
       </c>
       <c r="N113" t="n">
-        <v>927.6600000000001</v>
+        <v>927.66</v>
       </c>
     </row>
     <row r="114">
@@ -7557,7 +7557,7 @@
         </is>
       </c>
       <c r="N115" t="n">
-        <v>950.4000000000001</v>
+        <v>950.4</v>
       </c>
     </row>
     <row r="116">
@@ -8177,7 +8177,7 @@
         </is>
       </c>
       <c r="N125" t="n">
-        <v>834.1200000000001</v>
+        <v>834.12</v>
       </c>
     </row>
     <row r="126">
@@ -12331,7 +12331,7 @@
         </is>
       </c>
       <c r="N192" t="n">
-        <v>671.0999999999999</v>
+        <v>671.1</v>
       </c>
     </row>
     <row r="193">
@@ -13075,7 +13075,7 @@
         </is>
       </c>
       <c r="N204" t="n">
-        <v>761.9399999999999</v>
+        <v>761.9400000000001</v>
       </c>
     </row>
     <row r="205">
@@ -14501,7 +14501,7 @@
         </is>
       </c>
       <c r="N227" t="n">
-        <v>821.8799999999999</v>
+        <v>821.88</v>
       </c>
     </row>
     <row r="228">
@@ -16299,7 +16299,7 @@
         </is>
       </c>
       <c r="N256" t="n">
-        <v>789.5699999999999</v>
+        <v>789.5700000000001</v>
       </c>
     </row>
     <row r="257">
@@ -19771,7 +19771,7 @@
         </is>
       </c>
       <c r="N312" t="n">
-        <v>397.4399999999999</v>
+        <v>397.44</v>
       </c>
     </row>
     <row r="313">
@@ -22375,7 +22375,7 @@
         </is>
       </c>
       <c r="N354" t="n">
-        <v>869.8000000000001</v>
+        <v>869.8</v>
       </c>
     </row>
     <row r="355">
@@ -28389,7 +28389,7 @@
         </is>
       </c>
       <c r="N451" t="n">
-        <v>759.1500000000001</v>
+        <v>759.15</v>
       </c>
     </row>
     <row r="452">
@@ -32419,7 +32419,7 @@
         </is>
       </c>
       <c r="N516" t="n">
-        <v>912.4499999999999</v>
+        <v>912.45</v>
       </c>
     </row>
     <row r="517">
@@ -37255,7 +37255,7 @@
         </is>
       </c>
       <c r="N594" t="n">
-        <v>612.8100000000001</v>
+        <v>612.8099999999999</v>
       </c>
     </row>
     <row r="595">
@@ -37999,7 +37999,7 @@
         </is>
       </c>
       <c r="N606" t="n">
-        <v>97.85999999999999</v>
+        <v>97.86</v>
       </c>
     </row>
     <row r="607">
@@ -54553,7 +54553,7 @@
         </is>
       </c>
       <c r="N873" t="n">
-        <v>972.9000000000001</v>
+        <v>972.9</v>
       </c>
     </row>
     <row r="874">
@@ -54801,7 +54801,7 @@
         </is>
       </c>
       <c r="N877" t="n">
-        <v>666.9499999999999</v>
+        <v>666.95</v>
       </c>
     </row>
     <row r="878">
@@ -58707,7 +58707,7 @@
         </is>
       </c>
       <c r="N940" t="n">
-        <v>994.3799999999999</v>
+        <v>994.38</v>
       </c>
     </row>
     <row r="941">
@@ -61993,7 +61993,7 @@
         </is>
       </c>
       <c r="N993" t="n">
-        <v>635.9000000000001</v>
+        <v>635.9</v>
       </c>
     </row>
     <row r="994">
@@ -62117,7 +62117,7 @@
         </is>
       </c>
       <c r="N995" t="n">
-        <v>802.3499999999999</v>
+        <v>802.35</v>
       </c>
     </row>
     <row r="996">
@@ -63667,7 +63667,7 @@
         </is>
       </c>
       <c r="N1020" t="n">
-        <v>547.4399999999999</v>
+        <v>547.4400000000001</v>
       </c>
     </row>
     <row r="1021">
@@ -68193,7 +68193,7 @@
         </is>
       </c>
       <c r="N1093" t="n">
-        <v>628.4399999999999</v>
+        <v>628.4400000000001</v>
       </c>
     </row>
     <row r="1094">
@@ -69867,7 +69867,7 @@
         </is>
       </c>
       <c r="N1120" t="n">
-        <v>754.4399999999999</v>
+        <v>754.4400000000001</v>
       </c>
     </row>
     <row r="1121">
@@ -70363,7 +70363,7 @@
         </is>
       </c>
       <c r="N1128" t="n">
-        <v>950.5500000000001</v>
+        <v>950.55</v>
       </c>
     </row>
     <row r="1129">
@@ -72285,7 +72285,7 @@
         </is>
       </c>
       <c r="N1159" t="n">
-        <v>904.6500000000001</v>
+        <v>904.65</v>
       </c>
     </row>
     <row r="1160">
@@ -72657,7 +72657,7 @@
         </is>
       </c>
       <c r="N1165" t="n">
-        <v>918.8700000000001</v>
+        <v>918.87</v>
       </c>
     </row>
     <row r="1166">
@@ -72843,7 +72843,7 @@
         </is>
       </c>
       <c r="N1168" t="n">
-        <v>973.4100000000001</v>
+        <v>973.41</v>
       </c>
     </row>
     <row r="1169">
@@ -74579,7 +74579,7 @@
         </is>
       </c>
       <c r="N1196" t="n">
-        <v>568.3199999999999</v>
+        <v>568.3200000000001</v>
       </c>
     </row>
     <row r="1197">

</xml_diff>